<commit_message>
planning how to do the diagrams and and stuff moving forward in the NEA. currently in a dillema. do i use microsoft whiteboard or not? is it going to be sufficient? i guess ill find out.
</commit_message>
<xml_diff>
--- a/Filmtopia Checklist.xlsx
+++ b/Filmtopia Checklist.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mathe\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveholycrossac-my.sharepoint.com/personal/felixm25_holycross_ac_uk/Documents/Computer Science/NEA/FILMTOPIA/FILMTOPIA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3B493E5-65F9-4B31-A526-7E2C57131382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{E3B493E5-65F9-4B31-A526-7E2C57131382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2C6B9F1-85AC-4AE3-8AAB-F5903CABB6B6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -334,9 +334,6 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -348,6 +345,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -650,577 +650,577 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
+      <c r="B1" s="5"/>
     </row>
     <row r="3" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="str">
+      <c r="B3" s="2" t="str">
         <f>COUNTIF(B4:B13,"Done")&amp;"/"&amp;10</f>
         <v>10/10</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="str">
+      <c r="B14" s="2" t="str">
         <f>COUNTIF(B15:B28,"Done")&amp;"/"&amp;14</f>
         <v>14/14</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B28" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="2" t="s">
+      <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="3" t="str">
+      <c r="B29" s="2" t="str">
         <f>COUNTIF(B30:B40,"Done")&amp;"/"&amp;11</f>
-        <v>7/11</v>
+        <v>8/11</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B30" s="5" t="s">
-        <v>29</v>
+      <c r="B30" s="4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="B31" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="4" t="s">
+      <c r="A32" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="B33" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="4" t="s">
+      <c r="A34" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="B34" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="B35" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="4" t="s">
+      <c r="A36" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="B36" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="4" t="s">
+      <c r="A37" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="B37" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="4" t="s">
+      <c r="A38" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="B38" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="B39" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="B40" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="2" t="s">
+      <c r="A41" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B41" s="3" t="str">
+      <c r="B41" s="2" t="str">
         <f>COUNTIF(B42:B44,"Done")&amp;"/"&amp;3</f>
         <v>2/3</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="4" t="s">
+      <c r="A42" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="B42" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="4" t="s">
+      <c r="A43" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B43" s="5" t="s">
+      <c r="B43" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="4" t="s">
+      <c r="A44" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B44" s="5" t="s">
+      <c r="B44" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="2" t="s">
+      <c r="A45" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B45" s="3" t="str">
+      <c r="B45" s="2" t="str">
         <f>COUNTIF(B46:B50,"Done")&amp;"/"&amp;5</f>
         <v>0/5</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="4" t="s">
+      <c r="A46" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="B46" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="4" t="s">
+      <c r="A47" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B47" s="5" t="s">
+      <c r="B47" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="4" t="s">
+      <c r="A48" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B48" s="5" t="s">
+      <c r="B48" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="4" t="s">
+      <c r="A49" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="B49" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="4" t="s">
+      <c r="A50" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B50" s="5" t="s">
+      <c r="B50" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="2" t="s">
+      <c r="A51" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B51" s="3" t="str">
+      <c r="B51" s="2" t="str">
         <f>COUNTIF(B52:B58,"Done")&amp;"/"&amp;7</f>
         <v>0/7</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="4" t="s">
+      <c r="A52" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B52" s="5" t="s">
+      <c r="B52" s="4" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="4" t="s">
+      <c r="A53" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B53" s="5" t="s">
+      <c r="B53" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="4" t="s">
+      <c r="A54" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B54" s="5" t="s">
+      <c r="B54" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="4" t="s">
+      <c r="A55" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B55" s="5" t="s">
+      <c r="B55" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="4" t="s">
+      <c r="A56" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B56" s="5" t="s">
+      <c r="B56" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="4" t="s">
+      <c r="A57" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B57" s="5" t="s">
+      <c r="B57" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="4" t="s">
+      <c r="A58" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B58" s="5" t="s">
+      <c r="B58" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="2" t="s">
+      <c r="A59" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B59" s="3" t="str">
+      <c r="B59" s="2" t="str">
         <f>COUNTIF(B60:B60,"Done")&amp;"/"&amp;1</f>
         <v>0/1</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="4" t="s">
+      <c r="A60" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B60" s="5" t="s">
+      <c r="B60" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="2" t="s">
+      <c r="A61" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B61" s="3" t="str">
+      <c r="B61" s="2" t="str">
         <f>COUNTIF(B62:B64,"Done")&amp;"/"&amp;3</f>
         <v>2/3</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="4" t="s">
+      <c r="A62" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B62" s="5" t="s">
+      <c r="B62" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="4" t="s">
+      <c r="A63" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B63" s="5" t="s">
+      <c r="B63" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="4" t="s">
+      <c r="A64" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B64" s="5" t="s">
+      <c r="B64" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="2" t="s">
+      <c r="A65" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B65" s="3" t="str">
+      <c r="B65" s="2" t="str">
         <f>COUNTIF(B66:B72,"Done")&amp;"/"&amp;7</f>
         <v>0/7</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="4" t="s">
+      <c r="A66" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B66" s="5" t="s">
+      <c r="B66" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="4" t="s">
+      <c r="A67" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B67" s="5" t="s">
+      <c r="B67" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="4" t="s">
+      <c r="A68" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B68" s="5" t="s">
+      <c r="B68" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="4" t="s">
+      <c r="A69" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B69" s="5" t="s">
+      <c r="B69" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="4" t="s">
+      <c r="A70" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B70" s="5" t="s">
+      <c r="B70" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="4" t="s">
+      <c r="A71" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B71" s="5" t="s">
+      <c r="B71" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="4" t="s">
+      <c r="A72" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B72" s="5" t="s">
+      <c r="B72" s="4" t="s">
         <v>29</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added design for frmLogin in design
</commit_message>
<xml_diff>
--- a/Filmtopia Checklist.xlsx
+++ b/Filmtopia Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveholycrossac-my.sharepoint.com/personal/felixm25_holycross_ac_uk/Documents/Computer Science/NEA/FILMTOPIA/FILMTOPIA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{E3B493E5-65F9-4B31-A526-7E2C57131382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2C6B9F1-85AC-4AE3-8AAB-F5903CABB6B6}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{E3B493E5-65F9-4B31-A526-7E2C57131382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37368DDD-0984-433F-94F8-737B242CCFEB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -258,7 +258,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -299,8 +299,15 @@
       <name val="Arial"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B0F0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -319,6 +326,12 @@
         <bgColor rgb="FF993366"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -332,7 +345,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -349,6 +362,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -461,6 +475,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -642,7 +660,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B72"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="58" customWidth="1"/>
@@ -769,7 +787,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>15</v>
       </c>
@@ -777,7 +795,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>16</v>
       </c>
@@ -785,7 +803,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>17</v>
       </c>
@@ -793,7 +811,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
@@ -801,7 +819,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>19</v>
       </c>
@@ -809,7 +827,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>20</v>
       </c>
@@ -817,7 +835,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>21</v>
       </c>
@@ -825,7 +843,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>22</v>
       </c>
@@ -833,7 +851,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>23</v>
       </c>
@@ -841,7 +859,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>24</v>
       </c>
@@ -849,7 +867,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>25</v>
       </c>
@@ -857,7 +875,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>26</v>
       </c>
@@ -865,7 +883,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
@@ -874,7 +892,7 @@
         <v>8/11</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>28</v>
       </c>
@@ -882,21 +900,22 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
         <v>30</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
         <v>31</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>29</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="C32" s="6"/>
     </row>
     <row r="33" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">

</xml_diff>

<commit_message>
added design for frmFilms in design
</commit_message>
<xml_diff>
--- a/Filmtopia Checklist.xlsx
+++ b/Filmtopia Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveholycrossac-my.sharepoint.com/personal/felixm25_holycross_ac_uk/Documents/Computer Science/NEA/FILMTOPIA/FILMTOPIA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{E3B493E5-65F9-4B31-A526-7E2C57131382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37368DDD-0984-433F-94F8-737B242CCFEB}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{E3B493E5-65F9-4B31-A526-7E2C57131382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D0E4497-7C1F-4152-A419-9BE286E528A7}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -907,6 +907,7 @@
       <c r="B31" s="4" t="s">
         <v>52</v>
       </c>
+      <c r="C31" s="6"/>
     </row>
     <row r="32" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
@@ -915,7 +916,6 @@
       <c r="B32" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C32" s="6"/>
     </row>
     <row r="33" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">

</xml_diff>

<commit_message>
just added the form hierarchy diagram too
</commit_message>
<xml_diff>
--- a/Filmtopia Checklist.xlsx
+++ b/Filmtopia Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveholycrossac-my.sharepoint.com/personal/felixm25_holycross_ac_uk/Documents/Computer Science/NEA/FILMTOPIA/FILMTOPIA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{E3B493E5-65F9-4B31-A526-7E2C57131382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D0E4497-7C1F-4152-A419-9BE286E528A7}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{E3B493E5-65F9-4B31-A526-7E2C57131382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{419FF43B-53B1-4FDE-85E8-E8AF773C7609}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="74">
   <si>
     <t>FILMTOPIA — NEA CHECKLIST  (100 marks)</t>
   </si>
@@ -252,13 +252,19 @@
   </si>
   <si>
     <t>Potential Changes of Approach</t>
+  </si>
+  <si>
+    <t>kinda weird</t>
+  </si>
+  <si>
+    <t>just working on it now</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -306,8 +312,15 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -332,6 +345,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -345,7 +364,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -359,10 +378,14 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -660,7 +683,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:K72"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="58" customWidth="1"/>
@@ -668,10 +691,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
+      <c r="B1" s="6"/>
     </row>
     <row r="3" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -787,7 +810,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>15</v>
       </c>
@@ -795,7 +818,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>16</v>
       </c>
@@ -803,7 +826,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>17</v>
       </c>
@@ -811,7 +834,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
@@ -819,7 +842,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>19</v>
       </c>
@@ -827,7 +850,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>20</v>
       </c>
@@ -835,7 +858,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>21</v>
       </c>
@@ -843,7 +866,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>22</v>
       </c>
@@ -851,7 +874,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>23</v>
       </c>
@@ -859,7 +882,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>24</v>
       </c>
@@ -867,7 +890,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>25</v>
       </c>
@@ -875,7 +898,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>26</v>
       </c>
@@ -883,7 +906,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
@@ -892,30 +915,39 @@
         <v>8/11</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>28</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J30" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="K30" s="8"/>
+    </row>
+    <row r="31" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
         <v>30</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C31" s="6"/>
-    </row>
-    <row r="32" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C31" s="7"/>
+      <c r="J31" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="K31" s="10"/>
+    </row>
+    <row r="32" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
         <v>31</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>52</v>
       </c>
+      <c r="C32" s="5"/>
     </row>
     <row r="33" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
@@ -1047,7 +1079,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
         <v>48</v>
       </c>
@@ -1055,7 +1087,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
         <v>49</v>
       </c>
@@ -1063,7 +1095,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>50</v>
       </c>
@@ -1072,15 +1104,16 @@
         <v>0/7</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
         <v>51</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="53" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C52" s="8"/>
+    </row>
+    <row r="53" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
         <v>53</v>
       </c>
@@ -1088,7 +1121,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="54" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
         <v>54</v>
       </c>
@@ -1096,7 +1129,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="55" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
         <v>55</v>
       </c>
@@ -1104,7 +1137,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="3" t="s">
         <v>56</v>
       </c>
@@ -1112,7 +1145,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
         <v>57</v>
       </c>
@@ -1120,7 +1153,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="3" t="s">
         <v>58</v>
       </c>
@@ -1128,7 +1161,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="59" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>59</v>
       </c>
@@ -1137,7 +1170,7 @@
         <v>0/1</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="3" t="s">
         <v>60</v>
       </c>
@@ -1145,7 +1178,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="61" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>61</v>
       </c>
@@ -1154,7 +1187,7 @@
         <v>2/3</v>
       </c>
     </row>
-    <row r="62" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="3" t="s">
         <v>2</v>
       </c>
@@ -1162,7 +1195,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="63" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="3" t="s">
         <v>62</v>
       </c>
@@ -1170,7 +1203,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="64" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="3" t="s">
         <v>63</v>
       </c>

</xml_diff>

<commit_message>
key milestone: all work for prototype other than taking screenshots and summarising them is done. therefore gonna do a quick check through all of it to see how it holds up.
</commit_message>
<xml_diff>
--- a/Filmtopia Checklist.xlsx
+++ b/Filmtopia Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveholycrossac-my.sharepoint.com/personal/felixm25_holycross_ac_uk/Documents/Computer Science/NEA/FILMTOPIA/FILMTOPIA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="48" documentId="13_ncr:1_{E3B493E5-65F9-4B31-A526-7E2C57131382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{35E7D5AA-9C23-4B5D-8BEE-F8B18D40BFCF}"/>
+  <xr:revisionPtr revIDLastSave="53" documentId="13_ncr:1_{E3B493E5-65F9-4B31-A526-7E2C57131382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75472FA8-4C45-404A-AD72-CB96E94826B7}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -366,7 +366,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -387,7 +387,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -692,13 +691,13 @@
     <col min="2" max="2" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="9"/>
     </row>
-    <row r="3" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -707,110 +706,122 @@
         <v>10/10</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C4" s="7"/>
+    </row>
+    <row r="5" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="7"/>
+    </row>
+    <row r="6" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="7"/>
+    </row>
+    <row r="7" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C7" s="7"/>
+    </row>
+    <row r="8" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C8" s="7"/>
+    </row>
+    <row r="9" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C9" s="7"/>
+    </row>
+    <row r="10" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C10" s="7"/>
+    </row>
+    <row r="11" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C11" s="7"/>
+    </row>
+    <row r="12" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C12" s="7"/>
+    </row>
+    <row r="13" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C13" s="7"/>
+    </row>
+    <row r="14" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B14" s="2" t="str">
         <f>COUNTIF(B15:B28,"Done")&amp;"/"&amp;14</f>
-        <v>13/14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>14/14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C15" s="7"/>
+    </row>
+    <row r="16" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>3</v>
       </c>
+      <c r="C16" s="7"/>
     </row>
     <row r="17" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
@@ -819,6 +830,7 @@
       <c r="B17" s="4" t="s">
         <v>3</v>
       </c>
+      <c r="C17" s="7"/>
     </row>
     <row r="18" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
@@ -827,6 +839,7 @@
       <c r="B18" s="4" t="s">
         <v>3</v>
       </c>
+      <c r="C18" s="7"/>
     </row>
     <row r="19" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
@@ -835,15 +848,16 @@
       <c r="B19" s="4" t="s">
         <v>3</v>
       </c>
+      <c r="C19" s="7"/>
     </row>
     <row r="20" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C20" s="6"/>
+        <v>3</v>
+      </c>
+      <c r="C20" s="7"/>
     </row>
     <row r="21" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
@@ -852,6 +866,7 @@
       <c r="B21" s="4" t="s">
         <v>3</v>
       </c>
+      <c r="C21" s="7"/>
     </row>
     <row r="22" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
@@ -860,6 +875,7 @@
       <c r="B22" s="4" t="s">
         <v>3</v>
       </c>
+      <c r="C22" s="7"/>
     </row>
     <row r="23" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
@@ -868,6 +884,7 @@
       <c r="B23" s="4" t="s">
         <v>3</v>
       </c>
+      <c r="C23" s="7"/>
     </row>
     <row r="24" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
@@ -876,6 +893,7 @@
       <c r="B24" s="4" t="s">
         <v>3</v>
       </c>
+      <c r="C24" s="7"/>
     </row>
     <row r="25" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
@@ -884,6 +902,7 @@
       <c r="B25" s="4" t="s">
         <v>3</v>
       </c>
+      <c r="C25" s="7"/>
     </row>
     <row r="26" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
@@ -892,6 +911,7 @@
       <c r="B26" s="4" t="s">
         <v>3</v>
       </c>
+      <c r="C26" s="7"/>
     </row>
     <row r="27" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
@@ -900,6 +920,7 @@
       <c r="B27" s="4" t="s">
         <v>3</v>
       </c>
+      <c r="C27" s="7"/>
     </row>
     <row r="28" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
@@ -908,6 +929,7 @@
       <c r="B28" s="4" t="s">
         <v>3</v>
       </c>
+      <c r="C28" s="7"/>
     </row>
     <row r="29" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -1000,7 +1022,7 @@
       <c r="B37" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C37" s="10"/>
+      <c r="C37" s="7"/>
     </row>
     <row r="38" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
@@ -1059,8 +1081,9 @@
         <v>43</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>29</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="C44" s="6"/>
     </row>
     <row r="45" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">

</xml_diff>

<commit_message>
starting post prototype dev
</commit_message>
<xml_diff>
--- a/Filmtopia Checklist.xlsx
+++ b/Filmtopia Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveholycrossac-my.sharepoint.com/personal/felixm25_holycross_ac_uk/Documents/Computer Science/NEA/FILMTOPIA/FILMTOPIA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="13_ncr:1_{E3B493E5-65F9-4B31-A526-7E2C57131382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75472FA8-4C45-404A-AD72-CB96E94826B7}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="13_ncr:1_{E3B493E5-65F9-4B31-A526-7E2C57131382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23D3F918-1AE0-4AB5-ADC1-DB5F9E11B3AC}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -316,7 +316,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -353,6 +353,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -366,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -387,6 +393,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1057,7 +1064,7 @@
       </c>
       <c r="B41" s="2" t="str">
         <f>COUNTIF(B42:B44,"Done")&amp;"/"&amp;3</f>
-        <v>2/3</v>
+        <v>3/3</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1067,6 +1074,7 @@
       <c r="B42" s="4" t="s">
         <v>3</v>
       </c>
+      <c r="C42" s="7"/>
     </row>
     <row r="43" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
@@ -1075,15 +1083,16 @@
       <c r="B43" s="4" t="s">
         <v>3</v>
       </c>
+      <c r="C43" s="7"/>
     </row>
     <row r="44" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
         <v>43</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C44" s="6"/>
+        <v>3</v>
+      </c>
+      <c r="C44" s="7"/>
     </row>
     <row r="45" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
@@ -1093,6 +1102,7 @@
         <f>COUNTIF(B46:B50,"Done")&amp;"/"&amp;5</f>
         <v>0/5</v>
       </c>
+      <c r="C45" s="10"/>
     </row>
     <row r="46" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">

</xml_diff>

<commit_message>
adding new objectives for everything after the prototype into the investigation doc
</commit_message>
<xml_diff>
--- a/Filmtopia Checklist.xlsx
+++ b/Filmtopia Checklist.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveholycrossac-my.sharepoint.com/personal/felixm25_holycross_ac_uk/Documents/Computer Science/NEA/FILMTOPIA/FILMTOPIA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="13_ncr:1_{E3B493E5-65F9-4B31-A526-7E2C57131382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23D3F918-1AE0-4AB5-ADC1-DB5F9E11B3AC}"/>
+  <xr:revisionPtr revIDLastSave="61" documentId="13_ncr:1_{E3B493E5-65F9-4B31-A526-7E2C57131382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{21DA2750-E2AD-472F-ABDA-E2EEB4284FBA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="76">
   <si>
     <t>FILMTOPIA — NEA CHECKLIST  (100 marks)</t>
   </si>
@@ -261,6 +261,9 @@
   </si>
   <si>
     <t>Needs rechecking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
   </si>
 </sst>
 </file>
@@ -390,10 +393,10 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -699,10 +702,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9"/>
+      <c r="B1" s="10"/>
     </row>
     <row r="3" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -1102,14 +1105,14 @@
         <f>COUNTIF(B46:B50,"Done")&amp;"/"&amp;5</f>
         <v>0/5</v>
       </c>
-      <c r="C45" s="10"/>
+      <c r="C45" s="9"/>
     </row>
     <row r="46" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
         <v>45</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1117,7 +1120,10 @@
         <v>46</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>29</v>
+        <v>52</v>
+      </c>
+      <c r="C47" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1125,7 +1131,7 @@
         <v>47</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1133,7 +1139,7 @@
         <v>48</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1141,7 +1147,7 @@
         <v>49</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1338,7 +1344,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="B4:B13 B15:B28 B30:B40 B42:B44 B46:B50 B52:B58 B60 B62:B64 B66:B72" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="B4:B13 B15:B28 B30:B40 B42:B44 B66:B72 B52:B58 B60 B62:B64 B46:B50" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Not Started,In Progress,Done"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
fixed buying tickets on its own at kiosk
</commit_message>
<xml_diff>
--- a/Filmtopia Checklist.xlsx
+++ b/Filmtopia Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveholycrossac-my.sharepoint.com/personal/felixm25_holycross_ac_uk/Documents/Computer Science/NEA/FILMTOPIA/FILMTOPIA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="61" documentId="13_ncr:1_{E3B493E5-65F9-4B31-A526-7E2C57131382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{21DA2750-E2AD-472F-ABDA-E2EEB4284FBA}"/>
+  <xr:revisionPtr revIDLastSave="62" documentId="13_ncr:1_{E3B493E5-65F9-4B31-A526-7E2C57131382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{480847DA-FC6B-45F9-8D64-3EF5BCD2682E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1230,7 +1230,7 @@
         <v>60</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>